<commit_message>
MAJ pipeline 2026-07-30 10:04
</commit_message>
<xml_diff>
--- a/jira_export_2026-07-30.xlsx
+++ b/jira_export_2026-07-30.xlsx
@@ -723,7 +723,7 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>64,023 €</t>
+          <t>63,159 €</t>
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
@@ -737,7 +737,7 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>67.4%</t>
+          <t>66.5%</t>
         </is>
       </c>
       <c r="H7" s="7" t="n"/>
@@ -763,14 +763,14 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>23,404 €</t>
+          <t>23,600 €</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>40,619 €</t>
+          <t>39,559 €</t>
         </is>
       </c>
       <c r="E11" s="7" t="n"/>
@@ -818,7 +818,7 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>576 h</t>
+          <t>577 h</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -832,7 +832,7 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>68.6%</t>
+          <t>68.7%</t>
         </is>
       </c>
       <c r="H16" s="7" t="n"/>
@@ -903,7 +903,7 @@
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>257</t>
         </is>
       </c>
       <c r="H25" s="7" t="n"/>
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="N20" s="15" t="n">
-        <v>0</v>
+        <v>1660</v>
       </c>
       <c r="O20" s="15" t="n">
         <v>2075</v>
@@ -2400,10 +2400,10 @@
         <v>1296</v>
       </c>
       <c r="O23" s="12" t="n">
-        <v>2376</v>
+        <v>2448</v>
       </c>
       <c r="P23" s="12" t="n">
-        <v>153.29</v>
+        <v>157.94</v>
       </c>
     </row>
     <row r="24">
@@ -2895,11 +2895,11 @@
       <c r="N30" s="15" t="n">
         <v>353.5</v>
       </c>
-      <c r="O30" s="15" t="n">
-        <v>1060.5</v>
+      <c r="O30" s="16" t="n">
+        <v>0</v>
       </c>
       <c r="P30" s="15" t="n">
-        <v>2121</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3320,10 +3320,10 @@
         <v>1242.9</v>
       </c>
       <c r="O36" s="16" t="n">
-        <v>870.03</v>
+        <v>994.3200000000001</v>
       </c>
       <c r="P36" s="15" t="n">
-        <v>79.09</v>
+        <v>90.39</v>
       </c>
     </row>
     <row r="37">
@@ -12700,7 +12700,7 @@
         <v>27</v>
       </c>
       <c r="K169" s="11" t="n">
-        <v>1.75</v>
+        <v>2.5</v>
       </c>
       <c r="L169" s="11" t="inlineStr">
         <is>
@@ -13939,13 +13939,13 @@
       <c r="L190" s="17" t="inlineStr"/>
       <c r="M190" s="17" t="inlineStr"/>
       <c r="N190" s="18" t="n">
-        <v>62442.1</v>
+        <v>64102.1</v>
       </c>
       <c r="O190" s="18" t="n">
-        <v>64023.09500000001</v>
+        <v>63158.88500000001</v>
       </c>
       <c r="P190" s="18" t="n">
-        <v>182.66</v>
+        <v>179.81</v>
       </c>
     </row>
   </sheetData>
@@ -15163,7 +15163,7 @@
         </is>
       </c>
       <c r="B5" s="14" t="n">
-        <v>199.25</v>
+        <v>200</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>36</v>
@@ -15172,7 +15172,7 @@
         <v>4</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>239.25</v>
+        <v>240</v>
       </c>
       <c r="F5" s="14" t="n">
         <v>68.5</v>
@@ -15182,7 +15182,7 @@
       </c>
       <c r="H5" s="21" t="inlineStr">
         <is>
-          <t>49.2%</t>
+          <t>49.4%</t>
         </is>
       </c>
     </row>
@@ -15224,7 +15224,7 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>132.58</v>
+        <v>133.08</v>
       </c>
     </row>
   </sheetData>
@@ -15309,10 +15309,10 @@
         </is>
       </c>
       <c r="B5" s="24" t="n">
-        <v>387310</v>
+        <v>386693</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>129194</v>
+        <v>128576</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>258116</v>
@@ -15334,10 +15334,10 @@
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>175551</v>
+        <v>177055</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>70156</v>
+        <v>71660</v>
       </c>
       <c r="D6" s="25" t="n">
         <v>105395</v>
@@ -15359,10 +15359,10 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>211759</v>
+        <v>209638</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>59037</v>
+        <v>56916</v>
       </c>
       <c r="D7" s="26" t="n">
         <v>152722</v>
@@ -15388,7 +15388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15412,7 +15412,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Épics créées ce mois — 20 commande(s)</t>
+          <t>Épics créées ce mois — 21 commande(s)</t>
         </is>
       </c>
     </row>
@@ -15512,22 +15512,22 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34825</t>
+          <t>PDMDEP-34466</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34819</t>
+          <t>PDMDEP-34457</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Ville de Bourges</t>
+          <t>Commune de La Flèche</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -15547,22 +15547,22 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>00177218</t>
+          <t>00172594</t>
         </is>
       </c>
       <c r="I6" s="26" t="n">
-        <v>0</v>
+        <v>4475</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34791</t>
+          <t>PDMDEP-34825</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34782</t>
+          <t>PDMDEP-34819</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -15572,7 +15572,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>MAIRIE DE SAINT-ISMIER</t>
+          <t>Ville de Bourges</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -15582,7 +15582,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Nouveau déploiement</t>
+          <t>Migration</t>
         </is>
       </c>
       <c r="G7" s="14" t="inlineStr">
@@ -15592,32 +15592,32 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>00177122</t>
+          <t>00177218</t>
         </is>
       </c>
       <c r="I7" s="25" t="n">
-        <v>2146.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34466</t>
+          <t>PDMDEP-34791</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34457</t>
+          <t>PDMDEP-34782</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Commune de La Flèche</t>
+          <t>MAIRIE DE SAINT-ISMIER</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Nouveau déploiement</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
@@ -15637,32 +15637,32 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>00172594</t>
+          <t>00177122</t>
         </is>
       </c>
       <c r="I8" s="26" t="n">
-        <v>4475</v>
+        <v>2146.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34768</t>
+          <t>PDMDEP-34481</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34761</t>
+          <t>PDMDEP-34475</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DU PUY EN VELAY</t>
+          <t>Mairie de Pontcharra</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
@@ -15682,32 +15682,32 @@
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>00177029</t>
+          <t>00172611</t>
         </is>
       </c>
       <c r="I9" s="25" t="n">
-        <v>5585</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34481</t>
+          <t>PDMDEP-34768</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34475</t>
+          <t>PDMDEP-34761</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Mairie de Pontcharra</t>
+          <t>COMMUNE DU PUY EN VELAY</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -15727,11 +15727,11 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>00172611</t>
+          <t>00177029</t>
         </is>
       </c>
       <c r="I10" s="26" t="n">
-        <v>1050</v>
+        <v>5585</v>
       </c>
     </row>
     <row r="11">
@@ -16142,22 +16142,22 @@
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34852</t>
+          <t>PDMDEP-34499</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>PDMDEP-34848</t>
+          <t>PDMDEP-34495</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>07/07/2026</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>COMMUNE DE BRUAY LA BUISSIERE</t>
+          <t>COMMUNE DE CLICHY</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -16177,32 +16177,32 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>00177232</t>
+          <t>00172678</t>
         </is>
       </c>
       <c r="I20" s="26" t="n">
-        <v>0</v>
+        <v>4300</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34722</t>
+          <t>PDMDEP-34861</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34718</t>
+          <t>PDMDEP-34857</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>VILLE DE VILLEURBANNE</t>
+          <t>COMMUNE DE BIARRITZ</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
@@ -16222,11 +16222,11 @@
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>00176875</t>
+          <t>00177271</t>
         </is>
       </c>
       <c r="I21" s="25" t="n">
-        <v>2800</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="22">
@@ -16265,22 +16265,22 @@
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34499</t>
+          <t>PDMDEP-34852</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>PDMDEP-34495</t>
+          <t>PDMDEP-34848</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>07/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>COMMUNE DE CLICHY</t>
+          <t>COMMUNE DE BRUAY LA BUISSIERE</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
@@ -16300,83 +16300,107 @@
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>00172678</t>
+          <t>00177232</t>
         </is>
       </c>
       <c r="I23" s="25" t="n">
-        <v>4300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
+          <t>PDMDEP-34722</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>PDMDEP-34718</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>VILLE DE VILLEURBANNE</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>LITTERALIS</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Vente additionnelle</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>00176875</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="n">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
           <t>PDMDEP-34654</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>PDMDEP-34650</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>21/07/2026</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>DEPARTEMENT DE L AIN (CD 01)</t>
         </is>
       </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>LITTERALIS</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>Vente additionnelle</t>
         </is>
       </c>
-      <c r="G24" s="11" t="inlineStr">
+      <c r="G25" s="14" t="inlineStr">
         <is>
           <t>Services</t>
         </is>
       </c>
-      <c r="H24" s="11" t="inlineStr">
+      <c r="H25" s="14" t="inlineStr">
         <is>
           <t>00176582</t>
         </is>
       </c>
-      <c r="I24" s="26" t="n">
+      <c r="I25" s="25" t="n">
         <v>495</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="n"/>
-      <c r="C25" s="17" t="n"/>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="17" t="n"/>
-      <c r="G25" s="17" t="n"/>
-      <c r="H25" s="17" t="inlineStr">
-        <is>
-          <t>20 commande(s)</t>
-        </is>
-      </c>
-      <c r="I25" s="24" t="n">
-        <v>38784</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
         <is>
-          <t>dont Littéralis</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B26" s="17" t="n"/>
@@ -16387,17 +16411,17 @@
       <c r="G26" s="17" t="n"/>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>5 commande(s)</t>
+          <t>21 commande(s)</t>
         </is>
       </c>
       <c r="I26" s="24" t="n">
-        <v>8095</v>
+        <v>40484</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>dont GEODP</t>
+          <t>dont Littéralis</t>
         </is>
       </c>
       <c r="B27" s="17" t="n"/>
@@ -16408,10 +16432,31 @@
       <c r="G27" s="17" t="n"/>
       <c r="H27" s="17" t="inlineStr">
         <is>
+          <t>6 commande(s)</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="n">
+        <v>9795</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>dont GEODP</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17" t="n"/>
+      <c r="D28" s="17" t="n"/>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="17" t="n"/>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
           <t>15 commande(s)</t>
         </is>
       </c>
-      <c r="I27" s="24" t="n">
+      <c r="I28" s="24" t="n">
         <v>30689</v>
       </c>
     </row>

</xml_diff>